<commit_message>
added problems INIT: POW
</commit_message>
<xml_diff>
--- a/DSA_Roadmap_Java.xlsx
+++ b/DSA_Roadmap_Java.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nites\OneDrive\Documents\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF80A91-3D14-408D-AA3E-9D9C1DF067C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE093B6D-C1F7-4F67-8CDC-C41F13A36D14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="50">
   <si>
     <t>Module</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>Not Started</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -616,7 +619,7 @@
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -631,7 +634,7 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D3">
         <v>0</v>

</xml_diff>